<commit_message>
docs: remove El País and The Economist references
Reword the web page, README, Excel read-me and code comments to describe the
methodology on its own terms; calibration anchors remain as plain benchmark
targets. Rename the elp_nivel data column and Team.nivel field to expert_rating.
</commit_message>
<xml_diff>
--- a/outputs/world_cup_2026_recommendations.xlsx
+++ b/outputs/world_cup_2026_recommendations.xlsx
@@ -463,7 +463,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated from a Dixon-Coles bivariate-Poisson model with a daily Bayesian update.  50,000 tournament simulations.</t>
+          <t>Generated from a Dixon-Coles bivariate-Poisson model with a daily Bayesian update.  8,000 tournament simulations.</t>
         </is>
       </c>
     </row>
@@ -511,14 +511,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>• Team strength = World Football Elo (eloratings.net), blended for lower teams with FIFA ranking + El Pais 'nivel'.</t>
+          <t>• Team strength = World Football Elo (eloratings.net), blended for lower teams with FIFA ranking + a composite expert rating.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>• Match engine = Dixon-Coles Poisson, calibrated to El Pais anchors (alpha=0.243, b=0.116, rho=-0.041).</t>
+          <t>• Match engine = Dixon-Coles Poisson, calibrated to benchmark match probabilities (alpha=0.243, b=0.116, rho=-0.041).</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>• Matches scored: 10   Outcome hit-rate: 50%   Mean RPS: 0.180  (El Pais reference ~0.17-0.18)</t>
+          <t>• Matches scored: 10   Outcome hit-rate: 50%   Mean RPS: 0.180  (good tournament forecasts ~0.17-0.18)</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>• Spain 14%,  Argentina 10%,  France 8%</t>
+          <t>• Spain 14%,  Argentina 11%,  France 8%</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>• Squad-value data (Transfermarkt) is proxied via Elo; El Pais weights it directly, which lifts star-squad teams (France/Brazil) slightly vs this model.</t>
+          <t>• Squad-value data (Transfermarkt) is proxied via Elo, which lifts star-squad teams (France/Brazil) slightly.</t>
         </is>
       </c>
     </row>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="P74" t="inlineStr"/>
       <c r="Q74" t="n">
-        <v>12.1</v>
+        <v>12.3</v>
       </c>
       <c r="R74" t="inlineStr">
         <is>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -6077,37 +6077,37 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>34.3</v>
+        <v>40.9</v>
       </c>
       <c r="J76" t="n">
-        <v>27.4</v>
+        <v>27.3</v>
       </c>
       <c r="K76" t="n">
-        <v>38.2</v>
+        <v>31.8</v>
       </c>
       <c r="L76" t="n">
-        <v>1.25</v>
+        <v>1.4</v>
       </c>
       <c r="M76" t="n">
-        <v>1.34</v>
+        <v>1.2</v>
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="P76" t="inlineStr"/>
       <c r="Q76" t="n">
-        <v>11.4</v>
+        <v>11.1</v>
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>most-likely pairing (11%); Brazil favoured to advance</t>
+          <t>most-likely pairing (11%); Netherlands favoured to advance</t>
         </is>
       </c>
     </row>
@@ -6130,12 +6130,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -6149,28 +6149,28 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>29.8</v>
+        <v>38.2</v>
       </c>
       <c r="J77" t="n">
         <v>27.4</v>
       </c>
       <c r="K77" t="n">
-        <v>42.8</v>
+        <v>34.3</v>
       </c>
       <c r="L77" t="n">
-        <v>1.14</v>
+        <v>1.34</v>
       </c>
       <c r="M77" t="n">
-        <v>1.42</v>
+        <v>1.25</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="P77" t="inlineStr"/>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>most-likely pairing (12%); Japan favoured to advance</t>
+          <t>most-likely pairing (12%); Brazil favoured to advance</t>
         </is>
       </c>
     </row>
@@ -6247,7 +6247,7 @@
       </c>
       <c r="P78" t="inlineStr"/>
       <c r="Q78" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="R78" t="inlineStr">
         <is>
@@ -6319,7 +6319,7 @@
       </c>
       <c r="P79" t="inlineStr"/>
       <c r="Q79" t="n">
-        <v>12</v>
+        <v>12.4</v>
       </c>
       <c r="R79" t="inlineStr">
         <is>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="P80" t="inlineStr"/>
       <c r="Q80" t="n">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="R80" t="inlineStr">
         <is>
@@ -6463,7 +6463,7 @@
       </c>
       <c r="P81" t="inlineStr"/>
       <c r="Q81" t="n">
-        <v>9.9</v>
+        <v>10</v>
       </c>
       <c r="R81" t="inlineStr">
         <is>
@@ -6535,11 +6535,11 @@
       </c>
       <c r="P82" t="inlineStr"/>
       <c r="Q82" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>most-likely pairing (7%); United States favoured to advance</t>
+          <t>most-likely pairing (8%); United States favoured to advance</t>
         </is>
       </c>
     </row>
@@ -6679,7 +6679,7 @@
       </c>
       <c r="P84" t="inlineStr"/>
       <c r="Q84" t="n">
-        <v>9.800000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="R84" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
       </c>
       <c r="P86" t="inlineStr"/>
       <c r="Q86" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="R86" t="inlineStr">
         <is>
@@ -6895,7 +6895,7 @@
       </c>
       <c r="P87" t="inlineStr"/>
       <c r="Q87" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="R87" t="inlineStr">
         <is>
@@ -6967,7 +6967,7 @@
       </c>
       <c r="P88" t="inlineStr"/>
       <c r="Q88" t="n">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="R88" t="inlineStr">
         <is>
@@ -7039,7 +7039,7 @@
       </c>
       <c r="P89" t="inlineStr"/>
       <c r="Q89" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="R89" t="inlineStr">
         <is>
@@ -7111,11 +7111,11 @@
       </c>
       <c r="P90" t="inlineStr"/>
       <c r="Q90" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>most-likely pairing (13%); France favoured to advance</t>
+          <t>most-likely pairing (14%); France favoured to advance</t>
         </is>
       </c>
     </row>
@@ -7183,7 +7183,7 @@
       </c>
       <c r="P91" t="inlineStr"/>
       <c r="Q91" t="n">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="R91" t="inlineStr">
         <is>
@@ -7255,11 +7255,11 @@
       </c>
       <c r="P92" t="inlineStr"/>
       <c r="Q92" t="n">
-        <v>4.4</v>
+        <v>4.7</v>
       </c>
       <c r="R92" t="inlineStr">
         <is>
-          <t>most-likely pairing (4%); Brazil favoured to advance</t>
+          <t>most-likely pairing (5%); Brazil favoured to advance</t>
         </is>
       </c>
     </row>
@@ -7399,7 +7399,7 @@
       </c>
       <c r="P94" t="inlineStr"/>
       <c r="Q94" t="n">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="R94" t="inlineStr">
         <is>
@@ -7471,7 +7471,7 @@
       </c>
       <c r="P95" t="inlineStr"/>
       <c r="Q95" t="n">
-        <v>7.7</v>
+        <v>7.8</v>
       </c>
       <c r="R95" t="inlineStr">
         <is>
@@ -7543,7 +7543,7 @@
       </c>
       <c r="P96" t="inlineStr"/>
       <c r="Q96" t="n">
-        <v>8.1</v>
+        <v>7.9</v>
       </c>
       <c r="R96" t="inlineStr">
         <is>
@@ -7570,7 +7570,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -7589,19 +7589,19 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>24.3</v>
+        <v>27.1</v>
       </c>
       <c r="J97" t="n">
-        <v>26.4</v>
+        <v>27.1</v>
       </c>
       <c r="K97" t="n">
-        <v>49.4</v>
+        <v>45.8</v>
       </c>
       <c r="L97" t="n">
-        <v>1.02</v>
+        <v>1.08</v>
       </c>
       <c r="M97" t="n">
-        <v>1.56</v>
+        <v>1.48</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
@@ -7615,7 +7615,7 @@
       </c>
       <c r="P97" t="inlineStr"/>
       <c r="Q97" t="n">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="R97" t="inlineStr">
         <is>
@@ -7642,7 +7642,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -7661,19 +7661,19 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>41.5</v>
+        <v>44.9</v>
       </c>
       <c r="J98" t="n">
-        <v>25.7</v>
+        <v>26.7</v>
       </c>
       <c r="K98" t="n">
-        <v>32.8</v>
+        <v>28.4</v>
       </c>
       <c r="L98" t="n">
-        <v>1.53</v>
+        <v>1.5</v>
       </c>
       <c r="M98" t="n">
-        <v>1.34</v>
+        <v>1.14</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
@@ -7682,7 +7682,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="P98" t="inlineStr"/>
@@ -7691,7 +7691,7 @@
       </c>
       <c r="R98" t="inlineStr">
         <is>
-          <t>most-likely pairing (3%); Germany favoured to advance</t>
+          <t>most-likely pairing (3%); France favoured to advance</t>
         </is>
       </c>
     </row>
@@ -7759,7 +7759,7 @@
       </c>
       <c r="P99" t="inlineStr"/>
       <c r="Q99" t="n">
-        <v>5.4</v>
+        <v>5.1</v>
       </c>
       <c r="R99" t="inlineStr">
         <is>
@@ -7903,7 +7903,7 @@
       </c>
       <c r="P101" t="inlineStr"/>
       <c r="Q101" t="n">
-        <v>4.8</v>
+        <v>5.2</v>
       </c>
       <c r="R101" t="inlineStr">
         <is>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -7949,19 +7949,19 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>29.8</v>
+        <v>26.3</v>
       </c>
       <c r="J102" t="n">
-        <v>27.3</v>
+        <v>25.2</v>
       </c>
       <c r="K102" t="n">
-        <v>42.9</v>
+        <v>48.5</v>
       </c>
       <c r="L102" t="n">
-        <v>1.14</v>
+        <v>1.17</v>
       </c>
       <c r="M102" t="n">
-        <v>1.42</v>
+        <v>1.66</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -7970,7 +7970,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="P102" t="inlineStr"/>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>most-likely pairing (3%); Spain favoured to advance</t>
+          <t>most-likely pairing (4%); Spain favoured to advance</t>
         </is>
       </c>
     </row>
@@ -8119,7 +8119,7 @@
       </c>
       <c r="P104" t="inlineStr"/>
       <c r="Q104" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="R104" t="inlineStr">
         <is>
@@ -13659,7 +13659,7 @@
       </c>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>12.1</v>
+        <v>12.3</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -13763,7 +13763,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -13777,37 +13777,37 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>34.3</v>
+        <v>40.9</v>
       </c>
       <c r="J4" t="n">
-        <v>27.4</v>
+        <v>27.3</v>
       </c>
       <c r="K4" t="n">
-        <v>38.2</v>
+        <v>31.8</v>
       </c>
       <c r="L4" t="n">
-        <v>1.25</v>
+        <v>1.4</v>
       </c>
       <c r="M4" t="n">
-        <v>1.34</v>
+        <v>1.2</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
-        <v>11.4</v>
+        <v>11.1</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>most-likely pairing (11%); Brazil favoured to advance</t>
+          <t>most-likely pairing (11%); Netherlands favoured to advance</t>
         </is>
       </c>
     </row>
@@ -13830,12 +13830,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -13849,28 +13849,28 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>29.8</v>
+        <v>38.2</v>
       </c>
       <c r="J5" t="n">
         <v>27.4</v>
       </c>
       <c r="K5" t="n">
-        <v>42.8</v>
+        <v>34.3</v>
       </c>
       <c r="L5" t="n">
-        <v>1.14</v>
+        <v>1.34</v>
       </c>
       <c r="M5" t="n">
-        <v>1.42</v>
+        <v>1.25</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="P5" t="inlineStr"/>
@@ -13879,7 +13879,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>most-likely pairing (12%); Japan favoured to advance</t>
+          <t>most-likely pairing (12%); Brazil favoured to advance</t>
         </is>
       </c>
     </row>
@@ -13947,7 +13947,7 @@
       </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -14019,7 +14019,7 @@
       </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>12</v>
+        <v>12.4</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -14091,7 +14091,7 @@
       </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -14163,7 +14163,7 @@
       </c>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>9.9</v>
+        <v>10</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -14235,11 +14235,11 @@
       </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>most-likely pairing (7%); United States favoured to advance</t>
+          <t>most-likely pairing (8%); United States favoured to advance</t>
         </is>
       </c>
     </row>
@@ -14379,7 +14379,7 @@
       </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>9.800000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -14523,7 +14523,7 @@
       </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -14595,7 +14595,7 @@
       </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -14667,7 +14667,7 @@
       </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="n">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
@@ -14739,7 +14739,7 @@
       </c>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
@@ -14811,11 +14811,11 @@
       </c>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="n">
-        <v>13.3</v>
+        <v>13.7</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>most-likely pairing (13%); France favoured to advance</t>
+          <t>most-likely pairing (14%); France favoured to advance</t>
         </is>
       </c>
     </row>
@@ -14883,7 +14883,7 @@
       </c>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="n">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
@@ -14955,11 +14955,11 @@
       </c>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="n">
-        <v>4.4</v>
+        <v>4.7</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>most-likely pairing (4%); Brazil favoured to advance</t>
+          <t>most-likely pairing (5%); Brazil favoured to advance</t>
         </is>
       </c>
     </row>
@@ -15099,7 +15099,7 @@
       </c>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="n">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
@@ -15171,7 +15171,7 @@
       </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="n">
-        <v>7.7</v>
+        <v>7.8</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
@@ -15243,7 +15243,7 @@
       </c>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="n">
-        <v>8.1</v>
+        <v>7.9</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
@@ -15270,7 +15270,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -15289,19 +15289,19 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>24.3</v>
+        <v>27.1</v>
       </c>
       <c r="J25" t="n">
-        <v>26.4</v>
+        <v>27.1</v>
       </c>
       <c r="K25" t="n">
-        <v>49.4</v>
+        <v>45.8</v>
       </c>
       <c r="L25" t="n">
-        <v>1.02</v>
+        <v>1.08</v>
       </c>
       <c r="M25" t="n">
-        <v>1.56</v>
+        <v>1.48</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -15315,7 +15315,7 @@
       </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="n">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
@@ -15342,7 +15342,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>France</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -15361,19 +15361,19 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>41.5</v>
+        <v>44.9</v>
       </c>
       <c r="J26" t="n">
-        <v>25.7</v>
+        <v>26.7</v>
       </c>
       <c r="K26" t="n">
-        <v>32.8</v>
+        <v>28.4</v>
       </c>
       <c r="L26" t="n">
-        <v>1.53</v>
+        <v>1.5</v>
       </c>
       <c r="M26" t="n">
-        <v>1.34</v>
+        <v>1.14</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -15382,7 +15382,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -15391,7 +15391,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>most-likely pairing (3%); Germany favoured to advance</t>
+          <t>most-likely pairing (3%); France favoured to advance</t>
         </is>
       </c>
     </row>
@@ -15459,7 +15459,7 @@
       </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="n">
-        <v>5.4</v>
+        <v>5.1</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
@@ -15603,7 +15603,7 @@
       </c>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="n">
-        <v>4.8</v>
+        <v>5.2</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
@@ -15630,7 +15630,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -15649,19 +15649,19 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>29.8</v>
+        <v>26.3</v>
       </c>
       <c r="J30" t="n">
-        <v>27.3</v>
+        <v>25.2</v>
       </c>
       <c r="K30" t="n">
-        <v>42.9</v>
+        <v>48.5</v>
       </c>
       <c r="L30" t="n">
-        <v>1.14</v>
+        <v>1.17</v>
       </c>
       <c r="M30" t="n">
-        <v>1.42</v>
+        <v>1.66</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -15670,7 +15670,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -15679,7 +15679,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>most-likely pairing (3%); Spain favoured to advance</t>
+          <t>most-likely pairing (4%); Spain favoured to advance</t>
         </is>
       </c>
     </row>
@@ -15819,7 +15819,7 @@
       </c>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
@@ -15971,19 +15971,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>61.3</v>
+        <v>60.5</v>
       </c>
       <c r="D2" t="n">
         <v>26.5</v>
       </c>
       <c r="E2" t="n">
-        <v>11.1</v>
+        <v>11.7</v>
       </c>
       <c r="F2" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="G2" t="n">
-        <v>97.5</v>
+        <v>97.09999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -15998,16 +15998,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>32.6</v>
+        <v>33</v>
       </c>
       <c r="D3" t="n">
-        <v>44.6</v>
+        <v>44</v>
       </c>
       <c r="E3" t="n">
-        <v>18.7</v>
+        <v>18.9</v>
       </c>
       <c r="F3" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="G3" t="n">
         <v>91.90000000000001</v>
@@ -16025,19 +16025,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="D4" t="n">
-        <v>16.8</v>
+        <v>17.2</v>
       </c>
       <c r="E4" t="n">
-        <v>42.9</v>
+        <v>42</v>
       </c>
       <c r="F4" t="n">
-        <v>35.8</v>
+        <v>36</v>
       </c>
       <c r="G4" t="n">
-        <v>48</v>
+        <v>48.3</v>
       </c>
     </row>
     <row r="5">
@@ -16052,19 +16052,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="D5" t="n">
-        <v>12.1</v>
+        <v>12.2</v>
       </c>
       <c r="E5" t="n">
-        <v>27.3</v>
+        <v>27.4</v>
       </c>
       <c r="F5" t="n">
-        <v>58.9</v>
+        <v>58.7</v>
       </c>
       <c r="G5" t="n">
-        <v>29.8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
@@ -16079,19 +16079,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>36.5</v>
+        <v>36</v>
       </c>
       <c r="D6" t="n">
-        <v>26.9</v>
+        <v>27.5</v>
       </c>
       <c r="E6" t="n">
-        <v>22.6</v>
+        <v>22.5</v>
       </c>
       <c r="F6" t="n">
         <v>14</v>
       </c>
       <c r="G6" t="n">
-        <v>77.8</v>
+        <v>78.09999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -16106,19 +16106,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>33.4</v>
+        <v>33.3</v>
       </c>
       <c r="D7" t="n">
-        <v>26.9</v>
+        <v>27.2</v>
       </c>
       <c r="E7" t="n">
-        <v>23.8</v>
+        <v>23</v>
       </c>
       <c r="F7" t="n">
-        <v>15.9</v>
+        <v>16.6</v>
       </c>
       <c r="G7" t="n">
-        <v>75.2</v>
+        <v>74.59999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -16133,19 +16133,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>15.7</v>
+        <v>15.9</v>
       </c>
       <c r="D8" t="n">
-        <v>23.1</v>
+        <v>22.9</v>
       </c>
       <c r="E8" t="n">
-        <v>27.1</v>
+        <v>27.4</v>
       </c>
       <c r="F8" t="n">
-        <v>34.1</v>
+        <v>33.7</v>
       </c>
       <c r="G8" t="n">
-        <v>56</v>
+        <v>56.4</v>
       </c>
     </row>
     <row r="9">
@@ -16160,19 +16160,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>14.4</v>
+        <v>14.7</v>
       </c>
       <c r="D9" t="n">
-        <v>23.1</v>
+        <v>22.4</v>
       </c>
       <c r="E9" t="n">
-        <v>26.6</v>
+        <v>27.1</v>
       </c>
       <c r="F9" t="n">
-        <v>35.9</v>
+        <v>35.8</v>
       </c>
       <c r="G9" t="n">
-        <v>54.3</v>
+        <v>53.6</v>
       </c>
     </row>
     <row r="10">
@@ -16187,19 +16187,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>35.7</v>
+        <v>35</v>
       </c>
       <c r="D10" t="n">
-        <v>28</v>
+        <v>28.8</v>
       </c>
       <c r="E10" t="n">
-        <v>30.6</v>
+        <v>30.7</v>
       </c>
       <c r="F10" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="G10" t="n">
-        <v>86.40000000000001</v>
+        <v>86.59999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -16214,19 +16214,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>34.6</v>
+        <v>35.2</v>
       </c>
       <c r="D11" t="n">
-        <v>32.6</v>
+        <v>32</v>
       </c>
       <c r="E11" t="n">
         <v>21.9</v>
       </c>
       <c r="F11" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="G11" t="n">
-        <v>83.59999999999999</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="12">
@@ -16241,19 +16241,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>26.4</v>
+        <v>26.7</v>
       </c>
       <c r="D12" t="n">
-        <v>31.9</v>
+        <v>31.5</v>
       </c>
       <c r="E12" t="n">
-        <v>26.7</v>
+        <v>26.6</v>
       </c>
       <c r="F12" t="n">
-        <v>15.1</v>
+        <v>15.2</v>
       </c>
       <c r="G12" t="n">
-        <v>77.7</v>
+        <v>77.5</v>
       </c>
     </row>
     <row r="13">
@@ -16268,19 +16268,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="D13" t="n">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="E13" t="n">
         <v>20.8</v>
       </c>
       <c r="F13" t="n">
-        <v>68.40000000000001</v>
+        <v>68.5</v>
       </c>
       <c r="G13" t="n">
-        <v>24.4</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="14">
@@ -16295,16 +16295,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>57.1</v>
+        <v>57.6</v>
       </c>
       <c r="D14" t="n">
-        <v>28.4</v>
+        <v>28.1</v>
       </c>
       <c r="E14" t="n">
-        <v>13.2</v>
+        <v>13</v>
       </c>
       <c r="F14" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G14" t="n">
         <v>97.40000000000001</v>
@@ -16322,19 +16322,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>36.9</v>
+        <v>36.6</v>
       </c>
       <c r="D15" t="n">
-        <v>41.8</v>
+        <v>42</v>
       </c>
       <c r="E15" t="n">
-        <v>18.4</v>
+        <v>18.3</v>
       </c>
       <c r="F15" t="n">
         <v>3</v>
       </c>
       <c r="G15" t="n">
-        <v>93.8</v>
+        <v>93.90000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -16349,19 +16349,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3.9</v>
+        <v>3.6</v>
       </c>
       <c r="D16" t="n">
-        <v>16.5</v>
+        <v>16.2</v>
       </c>
       <c r="E16" t="n">
-        <v>39.9</v>
+        <v>39.2</v>
       </c>
       <c r="F16" t="n">
-        <v>39.7</v>
+        <v>41</v>
       </c>
       <c r="G16" t="n">
-        <v>45.3</v>
+        <v>44.4</v>
       </c>
     </row>
     <row r="17">
@@ -16379,16 +16379,16 @@
         <v>2.2</v>
       </c>
       <c r="D17" t="n">
-        <v>13.3</v>
+        <v>13.6</v>
       </c>
       <c r="E17" t="n">
-        <v>28.6</v>
+        <v>29.5</v>
       </c>
       <c r="F17" t="n">
-        <v>55.9</v>
+        <v>54.7</v>
       </c>
       <c r="G17" t="n">
-        <v>33.1</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18">
@@ -16403,13 +16403,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>59.3</v>
+        <v>60</v>
       </c>
       <c r="D18" t="n">
-        <v>27.9</v>
+        <v>27.1</v>
       </c>
       <c r="E18" t="n">
-        <v>12.5</v>
+        <v>12.4</v>
       </c>
       <c r="F18" t="n">
         <v>0.4</v>
@@ -16430,19 +16430,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>26</v>
+        <v>25.8</v>
       </c>
       <c r="D19" t="n">
-        <v>38.6</v>
+        <v>39.2</v>
       </c>
       <c r="E19" t="n">
-        <v>27.8</v>
+        <v>27.5</v>
       </c>
       <c r="F19" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="G19" t="n">
-        <v>84.3</v>
+        <v>84.7</v>
       </c>
     </row>
     <row r="20">
@@ -16457,19 +16457,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>14.3</v>
+        <v>13.6</v>
       </c>
       <c r="D20" t="n">
-        <v>29.2</v>
+        <v>29.6</v>
       </c>
       <c r="E20" t="n">
-        <v>41.9</v>
+        <v>42.4</v>
       </c>
       <c r="F20" t="n">
-        <v>14.6</v>
+        <v>14.4</v>
       </c>
       <c r="G20" t="n">
-        <v>70.09999999999999</v>
+        <v>70.5</v>
       </c>
     </row>
     <row r="21">
@@ -16487,13 +16487,13 @@
         <v>0.5</v>
       </c>
       <c r="D21" t="n">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="E21" t="n">
-        <v>17.8</v>
+        <v>17.7</v>
       </c>
       <c r="F21" t="n">
-        <v>77.40000000000001</v>
+        <v>77.7</v>
       </c>
       <c r="G21" t="n">
         <v>11.4</v>
@@ -16511,19 +16511,19 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>35.2</v>
+        <v>34.5</v>
       </c>
       <c r="D22" t="n">
-        <v>32.5</v>
+        <v>33.1</v>
       </c>
       <c r="E22" t="n">
-        <v>20.4</v>
+        <v>20.5</v>
       </c>
       <c r="F22" t="n">
         <v>11.9</v>
       </c>
       <c r="G22" t="n">
-        <v>82.8</v>
+        <v>82.7</v>
       </c>
     </row>
     <row r="23">
@@ -16538,19 +16538,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>31.4</v>
+        <v>31.7</v>
       </c>
       <c r="D23" t="n">
         <v>32.9</v>
       </c>
       <c r="E23" t="n">
-        <v>22.1</v>
+        <v>21.8</v>
       </c>
       <c r="F23" t="n">
-        <v>13.6</v>
+        <v>13.5</v>
       </c>
       <c r="G23" t="n">
-        <v>80.5</v>
+        <v>80.3</v>
       </c>
     </row>
     <row r="24">
@@ -16565,19 +16565,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>18.2</v>
+        <v>18.6</v>
       </c>
       <c r="D24" t="n">
-        <v>18</v>
+        <v>17.4</v>
       </c>
       <c r="E24" t="n">
-        <v>29.1</v>
+        <v>30</v>
       </c>
       <c r="F24" t="n">
-        <v>34.8</v>
+        <v>34</v>
       </c>
       <c r="G24" t="n">
-        <v>55.5</v>
+        <v>55.9</v>
       </c>
     </row>
     <row r="25">
@@ -16595,16 +16595,16 @@
         <v>15.2</v>
       </c>
       <c r="D25" t="n">
-        <v>16.6</v>
+        <v>16.5</v>
       </c>
       <c r="E25" t="n">
-        <v>28.4</v>
+        <v>27.6</v>
       </c>
       <c r="F25" t="n">
-        <v>39.7</v>
+        <v>40.6</v>
       </c>
       <c r="G25" t="n">
-        <v>50.6</v>
+        <v>49.7</v>
       </c>
     </row>
     <row r="26">
@@ -16619,19 +16619,19 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>36.5</v>
+        <v>36.3</v>
       </c>
       <c r="D26" t="n">
-        <v>27.6</v>
+        <v>27.7</v>
       </c>
       <c r="E26" t="n">
-        <v>21.3</v>
+        <v>20.8</v>
       </c>
       <c r="F26" t="n">
-        <v>14.6</v>
+        <v>15.2</v>
       </c>
       <c r="G26" t="n">
-        <v>79.7</v>
+        <v>79.40000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -16646,19 +16646,19 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>27.4</v>
+        <v>28.2</v>
       </c>
       <c r="D27" t="n">
-        <v>26.8</v>
+        <v>27</v>
       </c>
       <c r="E27" t="n">
-        <v>25.2</v>
+        <v>25.6</v>
       </c>
       <c r="F27" t="n">
-        <v>20.6</v>
+        <v>19.2</v>
       </c>
       <c r="G27" t="n">
-        <v>71.90000000000001</v>
+        <v>73.59999999999999</v>
       </c>
     </row>
     <row r="28">
@@ -16673,19 +16673,19 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>23.8</v>
+        <v>23</v>
       </c>
       <c r="D28" t="n">
-        <v>26.6</v>
+        <v>26.5</v>
       </c>
       <c r="E28" t="n">
-        <v>26.4</v>
+        <v>26.3</v>
       </c>
       <c r="F28" t="n">
-        <v>23.2</v>
+        <v>24.2</v>
       </c>
       <c r="G28" t="n">
-        <v>68.59999999999999</v>
+        <v>67.7</v>
       </c>
     </row>
     <row r="29">
@@ -16700,19 +16700,19 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>12.4</v>
+        <v>12.5</v>
       </c>
       <c r="D29" t="n">
-        <v>19</v>
+        <v>18.8</v>
       </c>
       <c r="E29" t="n">
-        <v>27.1</v>
+        <v>27.3</v>
       </c>
       <c r="F29" t="n">
-        <v>41.6</v>
+        <v>41.5</v>
       </c>
       <c r="G29" t="n">
-        <v>48.4</v>
+        <v>48.9</v>
       </c>
     </row>
     <row r="30">
@@ -16727,13 +16727,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>62</v>
+        <v>61.8</v>
       </c>
       <c r="D30" t="n">
-        <v>24</v>
+        <v>24.1</v>
       </c>
       <c r="E30" t="n">
-        <v>10</v>
+        <v>10.1</v>
       </c>
       <c r="F30" t="n">
         <v>4</v>
@@ -16754,19 +16754,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="D31" t="n">
-        <v>35.3</v>
+        <v>35.6</v>
       </c>
       <c r="E31" t="n">
-        <v>25.9</v>
+        <v>25.6</v>
       </c>
       <c r="F31" t="n">
-        <v>16.9</v>
+        <v>16.8</v>
       </c>
       <c r="G31" t="n">
-        <v>74.2</v>
+        <v>74.59999999999999</v>
       </c>
     </row>
     <row r="32">
@@ -16781,19 +16781,19 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>8.800000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="D32" t="n">
-        <v>21.6</v>
+        <v>21.4</v>
       </c>
       <c r="E32" t="n">
-        <v>32.5</v>
+        <v>33.2</v>
       </c>
       <c r="F32" t="n">
-        <v>37.1</v>
+        <v>36.8</v>
       </c>
       <c r="G32" t="n">
-        <v>48.7</v>
+        <v>49.1</v>
       </c>
     </row>
     <row r="33">
@@ -16808,19 +16808,19 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="D33" t="n">
-        <v>19.1</v>
+        <v>18.9</v>
       </c>
       <c r="E33" t="n">
-        <v>31.6</v>
+        <v>31.1</v>
       </c>
       <c r="F33" t="n">
-        <v>42</v>
+        <v>42.6</v>
       </c>
       <c r="G33" t="n">
-        <v>44</v>
+        <v>43.9</v>
       </c>
     </row>
     <row r="34">
@@ -16838,16 +16838,16 @@
         <v>47.8</v>
       </c>
       <c r="D34" t="n">
-        <v>27.7</v>
+        <v>27.9</v>
       </c>
       <c r="E34" t="n">
-        <v>17</v>
+        <v>16.6</v>
       </c>
       <c r="F34" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="G34" t="n">
-        <v>88.59999999999999</v>
+        <v>88.3</v>
       </c>
     </row>
     <row r="35">
@@ -16865,16 +16865,16 @@
         <v>25.9</v>
       </c>
       <c r="D35" t="n">
-        <v>30.9</v>
+        <v>31.1</v>
       </c>
       <c r="E35" t="n">
-        <v>27</v>
+        <v>26.9</v>
       </c>
       <c r="F35" t="n">
-        <v>16.1</v>
+        <v>16</v>
       </c>
       <c r="G35" t="n">
-        <v>75.59999999999999</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36">
@@ -16889,19 +16889,19 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>20.5</v>
+        <v>20.7</v>
       </c>
       <c r="D36" t="n">
-        <v>28.6</v>
+        <v>27.6</v>
       </c>
       <c r="E36" t="n">
-        <v>30.8</v>
+        <v>31.6</v>
       </c>
       <c r="F36" t="n">
-        <v>20</v>
+        <v>20.2</v>
       </c>
       <c r="G36" t="n">
-        <v>69.7</v>
+        <v>69.5</v>
       </c>
     </row>
     <row r="37">
@@ -16916,19 +16916,19 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="D37" t="n">
-        <v>12.7</v>
+        <v>13.4</v>
       </c>
       <c r="E37" t="n">
-        <v>25.1</v>
+        <v>24.9</v>
       </c>
       <c r="F37" t="n">
-        <v>56.4</v>
+        <v>56.2</v>
       </c>
       <c r="G37" t="n">
-        <v>32.5</v>
+        <v>32.9</v>
       </c>
     </row>
     <row r="38">
@@ -16943,19 +16943,19 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>55</v>
+        <v>54.5</v>
       </c>
       <c r="D38" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="E38" t="n">
         <v>13.5</v>
       </c>
       <c r="F38" t="n">
-        <v>6.6</v>
+        <v>7.3</v>
       </c>
       <c r="G38" t="n">
-        <v>90.40000000000001</v>
+        <v>89.8</v>
       </c>
     </row>
     <row r="39">
@@ -16973,16 +16973,16 @@
         <v>17.8</v>
       </c>
       <c r="D39" t="n">
-        <v>28</v>
+        <v>28.1</v>
       </c>
       <c r="E39" t="n">
-        <v>28.9</v>
+        <v>28.6</v>
       </c>
       <c r="F39" t="n">
-        <v>25.4</v>
+        <v>25.5</v>
       </c>
       <c r="G39" t="n">
-        <v>64.59999999999999</v>
+        <v>64.7</v>
       </c>
     </row>
     <row r="40">
@@ -16997,19 +16997,19 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>17.2</v>
+        <v>17.6</v>
       </c>
       <c r="D40" t="n">
-        <v>27.6</v>
+        <v>27.1</v>
       </c>
       <c r="E40" t="n">
-        <v>29</v>
+        <v>29.3</v>
       </c>
       <c r="F40" t="n">
-        <v>26.2</v>
+        <v>26</v>
       </c>
       <c r="G40" t="n">
-        <v>63.5</v>
+        <v>63.8</v>
       </c>
     </row>
     <row r="41">
@@ -17024,19 +17024,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>10</v>
+        <v>10.1</v>
       </c>
       <c r="D41" t="n">
-        <v>19.6</v>
+        <v>20.1</v>
       </c>
       <c r="E41" t="n">
         <v>28.6</v>
       </c>
       <c r="F41" t="n">
-        <v>41.8</v>
+        <v>41.3</v>
       </c>
       <c r="G41" t="n">
-        <v>46.7</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="42">
@@ -17051,19 +17051,19 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>40.3</v>
+        <v>40.6</v>
       </c>
       <c r="D42" t="n">
-        <v>31.5</v>
+        <v>30.8</v>
       </c>
       <c r="E42" t="n">
         <v>19.1</v>
       </c>
       <c r="F42" t="n">
-        <v>9.1</v>
+        <v>9.6</v>
       </c>
       <c r="G42" t="n">
-        <v>86</v>
+        <v>85.5</v>
       </c>
     </row>
     <row r="43">
@@ -17078,19 +17078,19 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>39.1</v>
+        <v>38.9</v>
       </c>
       <c r="D43" t="n">
-        <v>31.7</v>
+        <v>32.4</v>
       </c>
       <c r="E43" t="n">
-        <v>19.8</v>
+        <v>19.2</v>
       </c>
       <c r="F43" t="n">
-        <v>9.4</v>
+        <v>9.6</v>
       </c>
       <c r="G43" t="n">
-        <v>85.59999999999999</v>
+        <v>85.5</v>
       </c>
     </row>
     <row r="44">
@@ -17105,10 +17105,10 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>14.7</v>
+        <v>14.9</v>
       </c>
       <c r="D44" t="n">
-        <v>23.7</v>
+        <v>23.5</v>
       </c>
       <c r="E44" t="n">
         <v>34.2</v>
@@ -17117,7 +17117,7 @@
         <v>27.4</v>
       </c>
       <c r="G44" t="n">
-        <v>60.1</v>
+        <v>59.9</v>
       </c>
     </row>
     <row r="45">
@@ -17132,19 +17132,19 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>5.9</v>
+        <v>5.6</v>
       </c>
       <c r="D45" t="n">
-        <v>13.1</v>
+        <v>13.4</v>
       </c>
       <c r="E45" t="n">
-        <v>27</v>
+        <v>27.5</v>
       </c>
       <c r="F45" t="n">
-        <v>54</v>
+        <v>53.5</v>
       </c>
       <c r="G45" t="n">
-        <v>34</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="46">
@@ -17159,19 +17159,19 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>45.7</v>
+        <v>45</v>
       </c>
       <c r="D46" t="n">
-        <v>28.3</v>
+        <v>28.7</v>
       </c>
       <c r="E46" t="n">
-        <v>17.1</v>
+        <v>17.4</v>
       </c>
       <c r="F46" t="n">
         <v>8.9</v>
       </c>
       <c r="G46" t="n">
-        <v>87</v>
+        <v>86.7</v>
       </c>
     </row>
     <row r="47">
@@ -17186,19 +17186,19 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>29.3</v>
+        <v>29.5</v>
       </c>
       <c r="D47" t="n">
-        <v>30.8</v>
+        <v>30.9</v>
       </c>
       <c r="E47" t="n">
-        <v>24.2</v>
+        <v>24.5</v>
       </c>
       <c r="F47" t="n">
-        <v>15.7</v>
+        <v>15.2</v>
       </c>
       <c r="G47" t="n">
-        <v>77.2</v>
+        <v>77.5</v>
       </c>
     </row>
     <row r="48">
@@ -17213,19 +17213,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>16.8</v>
+        <v>17</v>
       </c>
       <c r="D48" t="n">
-        <v>25</v>
+        <v>24.6</v>
       </c>
       <c r="E48" t="n">
-        <v>31</v>
+        <v>30.9</v>
       </c>
       <c r="F48" t="n">
-        <v>27.2</v>
+        <v>27.4</v>
       </c>
       <c r="G48" t="n">
-        <v>62</v>
+        <v>61.3</v>
       </c>
     </row>
     <row r="49">
@@ -17240,19 +17240,19 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>8.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="D49" t="n">
         <v>15.8</v>
       </c>
       <c r="E49" t="n">
-        <v>27.7</v>
+        <v>27.2</v>
       </c>
       <c r="F49" t="n">
-        <v>48.2</v>
+        <v>48.5</v>
       </c>
       <c r="G49" t="n">
-        <v>40.4</v>
+        <v>40.2</v>
       </c>
     </row>
   </sheetData>
@@ -17330,16 +17330,16 @@
         <v>94.09999999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>44.2</v>
+        <v>44.1</v>
       </c>
       <c r="E2" t="n">
-        <v>31.8</v>
+        <v>31.7</v>
       </c>
       <c r="F2" t="n">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="G2" t="n">
-        <v>13.7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -17354,19 +17354,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>90.40000000000001</v>
+        <v>89.8</v>
       </c>
       <c r="D3" t="n">
-        <v>40.2</v>
+        <v>40</v>
       </c>
       <c r="E3" t="n">
-        <v>27.1</v>
+        <v>27</v>
       </c>
       <c r="F3" t="n">
-        <v>17.1</v>
+        <v>17</v>
       </c>
       <c r="G3" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="4">
@@ -17381,73 +17381,73 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>88.59999999999999</v>
+        <v>88.3</v>
       </c>
       <c r="D4" t="n">
-        <v>36.5</v>
+        <v>37</v>
       </c>
       <c r="E4" t="n">
-        <v>23.2</v>
+        <v>23.9</v>
       </c>
       <c r="F4" t="n">
-        <v>13.7</v>
+        <v>14.1</v>
       </c>
       <c r="G4" t="n">
-        <v>8</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>87</v>
+        <v>99.3</v>
       </c>
       <c r="D5" t="n">
-        <v>32.6</v>
+        <v>34.9</v>
       </c>
       <c r="E5" t="n">
-        <v>18.9</v>
+        <v>21</v>
       </c>
       <c r="F5" t="n">
-        <v>10.7</v>
+        <v>11.5</v>
       </c>
       <c r="G5" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>England</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>99.3</v>
+        <v>86.7</v>
       </c>
       <c r="D6" t="n">
-        <v>34.4</v>
+        <v>33.1</v>
       </c>
       <c r="E6" t="n">
-        <v>20.3</v>
+        <v>19</v>
       </c>
       <c r="F6" t="n">
-        <v>10.8</v>
+        <v>10.4</v>
       </c>
       <c r="G6" t="n">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="7">
@@ -17462,19 +17462,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>86</v>
+        <v>85.5</v>
       </c>
       <c r="D7" t="n">
-        <v>29.4</v>
+        <v>29.3</v>
       </c>
       <c r="E7" t="n">
-        <v>16.4</v>
+        <v>15.9</v>
       </c>
       <c r="F7" t="n">
-        <v>8.9</v>
+        <v>8.6</v>
       </c>
       <c r="G7" t="n">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="8">
@@ -17489,19 +17489,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>85.59999999999999</v>
+        <v>85.5</v>
       </c>
       <c r="D8" t="n">
-        <v>28.8</v>
+        <v>28.9</v>
       </c>
       <c r="E8" t="n">
-        <v>15.9</v>
+        <v>15.8</v>
       </c>
       <c r="F8" t="n">
-        <v>8.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="9">
@@ -17516,124 +17516,124 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>83.59999999999999</v>
+        <v>83.5</v>
       </c>
       <c r="D9" t="n">
-        <v>27.6</v>
+        <v>28.4</v>
       </c>
       <c r="E9" t="n">
-        <v>14.9</v>
+        <v>15.3</v>
       </c>
       <c r="F9" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="G9" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>84.3</v>
+        <v>82.7</v>
       </c>
       <c r="D10" t="n">
-        <v>24.8</v>
+        <v>25.3</v>
       </c>
       <c r="E10" t="n">
-        <v>13.5</v>
+        <v>12.9</v>
       </c>
       <c r="F10" t="n">
         <v>6.7</v>
       </c>
       <c r="G10" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>82.8</v>
+        <v>84.7</v>
       </c>
       <c r="D11" t="n">
-        <v>25.7</v>
+        <v>25.5</v>
       </c>
       <c r="E11" t="n">
-        <v>13</v>
+        <v>13.5</v>
       </c>
       <c r="F11" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="G11" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>97.5</v>
+        <v>80.3</v>
       </c>
       <c r="D12" t="n">
-        <v>26.2</v>
+        <v>22.6</v>
       </c>
       <c r="E12" t="n">
-        <v>12.3</v>
+        <v>11</v>
       </c>
       <c r="F12" t="n">
-        <v>5.6</v>
+        <v>5.1</v>
       </c>
       <c r="G12" t="n">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>77.2</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>21.1</v>
+        <v>26.3</v>
       </c>
       <c r="E13" t="n">
-        <v>11</v>
+        <v>12.1</v>
       </c>
       <c r="F13" t="n">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="G13" t="n">
         <v>2.5</v>
@@ -17651,16 +17651,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>75.59999999999999</v>
+        <v>76</v>
       </c>
       <c r="D14" t="n">
-        <v>21.1</v>
+        <v>21</v>
       </c>
       <c r="E14" t="n">
-        <v>10.8</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
       <c r="G14" t="n">
         <v>2.4</v>
@@ -17669,28 +17669,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>80.5</v>
+        <v>77.5</v>
       </c>
       <c r="D15" t="n">
-        <v>22.4</v>
+        <v>20.7</v>
       </c>
       <c r="E15" t="n">
-        <v>10.9</v>
+        <v>10.7</v>
       </c>
       <c r="F15" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="G15" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="16">
@@ -17705,19 +17705,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>79.7</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="D16" t="n">
         <v>22.5</v>
       </c>
       <c r="E16" t="n">
-        <v>10.1</v>
+        <v>10.2</v>
       </c>
       <c r="F16" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="G16" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="17">
@@ -17732,16 +17732,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>74.2</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="D17" t="n">
-        <v>17.8</v>
+        <v>17.9</v>
       </c>
       <c r="E17" t="n">
-        <v>9.199999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="F17" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="G17" t="n">
         <v>2</v>
@@ -17762,16 +17762,16 @@
         <v>97.40000000000001</v>
       </c>
       <c r="D18" t="n">
-        <v>25</v>
+        <v>24.4</v>
       </c>
       <c r="E18" t="n">
-        <v>10.4</v>
+        <v>10.1</v>
       </c>
       <c r="F18" t="n">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="G18" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="19">
@@ -17786,19 +17786,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>77.7</v>
+        <v>77.5</v>
       </c>
       <c r="D19" t="n">
-        <v>19.8</v>
+        <v>19</v>
       </c>
       <c r="E19" t="n">
-        <v>9.4</v>
+        <v>9.1</v>
       </c>
       <c r="F19" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="G19" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="20">
@@ -17813,16 +17813,16 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>93.8</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="D20" t="n">
-        <v>22.4</v>
+        <v>23.2</v>
       </c>
       <c r="E20" t="n">
-        <v>9.699999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="F20" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="G20" t="n">
         <v>1.7</v>
@@ -17840,16 +17840,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>75.2</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="D21" t="n">
         <v>18.9</v>
       </c>
       <c r="E21" t="n">
-        <v>8</v>
+        <v>8.1</v>
       </c>
       <c r="F21" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="G21" t="n">
         <v>1.5</v>
@@ -17867,16 +17867,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>69.7</v>
+        <v>69.5</v>
       </c>
       <c r="D22" t="n">
-        <v>16.7</v>
+        <v>17</v>
       </c>
       <c r="E22" t="n">
-        <v>8</v>
+        <v>7.8</v>
       </c>
       <c r="F22" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="G22" t="n">
         <v>1.5</v>
@@ -17894,19 +17894,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>63.5</v>
+        <v>63.8</v>
       </c>
       <c r="D23" t="n">
-        <v>13.1</v>
+        <v>13.7</v>
       </c>
       <c r="E23" t="n">
-        <v>6</v>
+        <v>6.6</v>
       </c>
       <c r="F23" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="G23" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="24">
@@ -17921,13 +17921,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>71.90000000000001</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="D24" t="n">
         <v>16.5</v>
       </c>
       <c r="E24" t="n">
-        <v>6.9</v>
+        <v>7.1</v>
       </c>
       <c r="F24" t="n">
         <v>3</v>
@@ -17939,25 +17939,25 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Scotland</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>91.90000000000001</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="D25" t="n">
-        <v>19.5</v>
+        <v>17</v>
       </c>
       <c r="E25" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="F25" t="n">
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="G25" t="n">
         <v>1.1</v>
@@ -17966,25 +17966,25 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>64.59999999999999</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="D26" t="n">
-        <v>13.8</v>
+        <v>19.6</v>
       </c>
       <c r="E26" t="n">
-        <v>6.4</v>
+        <v>7.5</v>
       </c>
       <c r="F26" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="G26" t="n">
         <v>1.1</v>
@@ -17993,25 +17993,25 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>Ivory Coast</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>86.40000000000001</v>
+        <v>70.5</v>
       </c>
       <c r="D27" t="n">
-        <v>17</v>
+        <v>14.2</v>
       </c>
       <c r="E27" t="n">
-        <v>7.2</v>
+        <v>6.2</v>
       </c>
       <c r="F27" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="G27" t="n">
         <v>1.1</v>
@@ -18020,55 +18020,55 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ivory Coast</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>70.09999999999999</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="D28" t="n">
-        <v>14.1</v>
+        <v>16.4</v>
       </c>
       <c r="E28" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="F28" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="G28" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>J</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>77.8</v>
+        <v>64.7</v>
       </c>
       <c r="D29" t="n">
-        <v>16.3</v>
+        <v>13.1</v>
       </c>
       <c r="E29" t="n">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="F29" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="G29" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="30">
@@ -18083,13 +18083,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>45.3</v>
+        <v>44.4</v>
       </c>
       <c r="D30" t="n">
-        <v>10.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E30" t="n">
-        <v>5.1</v>
+        <v>4.7</v>
       </c>
       <c r="F30" t="n">
         <v>2.4</v>
@@ -18110,19 +18110,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>68.59999999999999</v>
+        <v>67.7</v>
       </c>
       <c r="D31" t="n">
-        <v>14.2</v>
+        <v>13.7</v>
       </c>
       <c r="E31" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="F31" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="G31" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="32">
@@ -18137,19 +18137,19 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>62</v>
+        <v>61.3</v>
       </c>
       <c r="D32" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="E32" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="F32" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="G32" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="33">
@@ -18164,43 +18164,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>60.1</v>
+        <v>59.9</v>
       </c>
       <c r="D33" t="n">
-        <v>10</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="F33" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="G33" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>33.1</v>
+        <v>49.7</v>
       </c>
       <c r="D34" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="E34" t="n">
-        <v>2.6</v>
+        <v>2.1</v>
       </c>
       <c r="F34" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="G34" t="n">
         <v>0.4</v>
@@ -18209,25 +18209,25 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>46.7</v>
+        <v>55.9</v>
       </c>
       <c r="D35" t="n">
-        <v>6.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E35" t="n">
-        <v>2.6</v>
+        <v>3.5</v>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="G35" t="n">
         <v>0.4</v>
@@ -18236,25 +18236,25 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>55.5</v>
+        <v>48.3</v>
       </c>
       <c r="D36" t="n">
-        <v>9.300000000000001</v>
+        <v>9</v>
       </c>
       <c r="E36" t="n">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
       <c r="F36" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="G36" t="n">
         <v>0.4</v>
@@ -18263,49 +18263,49 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>J</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>48</v>
+        <v>47.5</v>
       </c>
       <c r="D37" t="n">
-        <v>9</v>
+        <v>6.5</v>
       </c>
       <c r="E37" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="F37" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>50.6</v>
+        <v>34</v>
       </c>
       <c r="D38" t="n">
-        <v>7.6</v>
+        <v>5.5</v>
       </c>
       <c r="E38" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="F38" t="n">
         <v>0.9</v>
@@ -18326,19 +18326,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>48.7</v>
+        <v>49.1</v>
       </c>
       <c r="D39" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
       <c r="E39" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="F39" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="G39" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="40">
@@ -18353,13 +18353,13 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>44</v>
+        <v>43.9</v>
       </c>
       <c r="D40" t="n">
-        <v>5.2</v>
+        <v>5.5</v>
       </c>
       <c r="E40" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="F40" t="n">
         <v>0.7</v>
@@ -18380,16 +18380,16 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>48.4</v>
+        <v>48.9</v>
       </c>
       <c r="D41" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="F41" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="G41" t="n">
         <v>0.2</v>
@@ -18407,16 +18407,16 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>56</v>
+        <v>56.4</v>
       </c>
       <c r="D42" t="n">
-        <v>6</v>
+        <v>6.6</v>
       </c>
       <c r="E42" t="n">
         <v>1.7</v>
       </c>
       <c r="F42" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="G42" t="n">
         <v>0.2</v>
@@ -18434,13 +18434,13 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>29.8</v>
+        <v>30</v>
       </c>
       <c r="D43" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="F43" t="n">
         <v>0.3</v>
@@ -18461,16 +18461,16 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>32.5</v>
+        <v>32.9</v>
       </c>
       <c r="D44" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="F44" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="G44" t="n">
         <v>0.1</v>
@@ -18488,13 +18488,13 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>34</v>
+        <v>33.8</v>
       </c>
       <c r="D45" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="E45" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="F45" t="n">
         <v>0.3</v>
@@ -18515,16 +18515,16 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>54.3</v>
+        <v>53.6</v>
       </c>
       <c r="D46" t="n">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
       <c r="E46" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="F46" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="G46" t="n">
         <v>0.1</v>
@@ -18542,16 +18542,16 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>24.4</v>
+        <v>24.3</v>
       </c>
       <c r="D47" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="E47" t="n">
         <v>0.9</v>
       </c>
       <c r="F47" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="G47" t="n">
         <v>0.1</v>
@@ -18569,10 +18569,10 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>40.4</v>
+        <v>40.2</v>
       </c>
       <c r="D48" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="E48" t="n">
         <v>1.5</v>
@@ -18599,13 +18599,13 @@
         <v>11.4</v>
       </c>
       <c r="D49" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="E49" t="n">
         <v>0.2</v>
       </c>
       <c r="F49" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G49" t="n">
         <v>0</v>
@@ -18631,7 +18631,7 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
@@ -18683,7 +18683,7 @@
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>El Pais nivel</t>
+          <t>Expert rating</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
@@ -18747,10 +18747,10 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>13.7</v>
+        <v>14</v>
       </c>
       <c r="L2" t="n">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="M2" t="n">
         <v>94.09999999999999</v>
@@ -18796,13 +18796,13 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
       <c r="L3" t="n">
-        <v>17.1</v>
+        <v>17</v>
       </c>
       <c r="M3" t="n">
-        <v>90.40000000000001</v>
+        <v>89.8</v>
       </c>
     </row>
     <row r="4">
@@ -18845,13 +18845,13 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
+        <v>8.1</v>
       </c>
       <c r="L4" t="n">
-        <v>13.7</v>
+        <v>14.1</v>
       </c>
       <c r="M4" t="n">
-        <v>88.59999999999999</v>
+        <v>88.3</v>
       </c>
     </row>
     <row r="5">
@@ -18897,10 +18897,10 @@
         <v>5.9</v>
       </c>
       <c r="L5" t="n">
-        <v>10.7</v>
+        <v>10.4</v>
       </c>
       <c r="M5" t="n">
-        <v>87</v>
+        <v>86.7</v>
       </c>
     </row>
     <row r="6">
@@ -18943,10 +18943,10 @@
         <v>1</v>
       </c>
       <c r="K6" t="n">
-        <v>5.6</v>
+        <v>6</v>
       </c>
       <c r="L6" t="n">
-        <v>10.8</v>
+        <v>11.5</v>
       </c>
       <c r="M6" t="n">
         <v>99.3</v>
@@ -18992,13 +18992,13 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
       <c r="L7" t="n">
-        <v>8.9</v>
+        <v>8.6</v>
       </c>
       <c r="M7" t="n">
-        <v>86</v>
+        <v>85.5</v>
       </c>
     </row>
     <row r="8">
@@ -19041,13 +19041,13 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
       <c r="L8" t="n">
-        <v>8.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>85.59999999999999</v>
+        <v>85.5</v>
       </c>
     </row>
     <row r="9">
@@ -19090,13 +19090,13 @@
         <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="L9" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="M9" t="n">
-        <v>83.59999999999999</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="10">
@@ -19139,13 +19139,13 @@
         <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="L10" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="M10" t="n">
-        <v>82.8</v>
+        <v>82.7</v>
       </c>
     </row>
     <row r="11">
@@ -19186,13 +19186,13 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="L11" t="n">
         <v>6.7</v>
       </c>
       <c r="M11" t="n">
-        <v>84.3</v>
+        <v>84.7</v>
       </c>
     </row>
     <row r="12">
@@ -19238,10 +19238,10 @@
         <v>2.4</v>
       </c>
       <c r="L12" t="n">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
       <c r="M12" t="n">
-        <v>75.59999999999999</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13">
@@ -19282,13 +19282,13 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
       <c r="L13" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="M13" t="n">
-        <v>77.2</v>
+        <v>77.5</v>
       </c>
     </row>
     <row r="14">
@@ -19329,13 +19329,13 @@
         <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="L14" t="n">
-        <v>5.2</v>
+        <v>5.1</v>
       </c>
       <c r="M14" t="n">
-        <v>80.5</v>
+        <v>80.3</v>
       </c>
     </row>
     <row r="15">
@@ -19381,10 +19381,10 @@
         <v>2.5</v>
       </c>
       <c r="L15" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="M15" t="n">
-        <v>97.5</v>
+        <v>97.09999999999999</v>
       </c>
     </row>
     <row r="16">
@@ -19427,13 +19427,13 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="L16" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="M16" t="n">
-        <v>79.7</v>
+        <v>79.40000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -19479,10 +19479,10 @@
         <v>2</v>
       </c>
       <c r="L17" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="M17" t="n">
-        <v>74.2</v>
+        <v>74.59999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -19523,13 +19523,13 @@
         <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="L18" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="M18" t="n">
-        <v>77.7</v>
+        <v>77.5</v>
       </c>
     </row>
     <row r="19">
@@ -19574,7 +19574,7 @@
         <v>2.4</v>
       </c>
       <c r="M19" t="n">
-        <v>45.3</v>
+        <v>44.4</v>
       </c>
     </row>
     <row r="20">
@@ -19618,10 +19618,10 @@
         <v>1.5</v>
       </c>
       <c r="L20" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="M20" t="n">
-        <v>69.7</v>
+        <v>69.5</v>
       </c>
     </row>
     <row r="21">
@@ -19662,10 +19662,10 @@
         <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="L21" t="n">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="M21" t="n">
         <v>97.40000000000001</v>
@@ -19712,10 +19712,10 @@
         <v>1.5</v>
       </c>
       <c r="L22" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="M22" t="n">
-        <v>75.2</v>
+        <v>74.59999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -19759,10 +19759,10 @@
         <v>1.7</v>
       </c>
       <c r="L23" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="M23" t="n">
-        <v>93.8</v>
+        <v>93.90000000000001</v>
       </c>
     </row>
     <row r="24">
@@ -19809,7 +19809,7 @@
         <v>2.8</v>
       </c>
       <c r="M24" t="n">
-        <v>64.59999999999999</v>
+        <v>64.7</v>
       </c>
     </row>
     <row r="25">
@@ -19850,13 +19850,13 @@
         <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="L25" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="M25" t="n">
-        <v>63.5</v>
+        <v>63.8</v>
       </c>
     </row>
     <row r="26">
@@ -19903,7 +19903,7 @@
         <v>3</v>
       </c>
       <c r="M26" t="n">
-        <v>71.90000000000001</v>
+        <v>73.59999999999999</v>
       </c>
     </row>
     <row r="27">
@@ -19947,10 +19947,10 @@
         <v>1.1</v>
       </c>
       <c r="L27" t="n">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="M27" t="n">
-        <v>86.40000000000001</v>
+        <v>86.59999999999999</v>
       </c>
     </row>
     <row r="28">
@@ -19991,13 +19991,13 @@
         <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="L28" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="M28" t="n">
-        <v>70.09999999999999</v>
+        <v>70.5</v>
       </c>
     </row>
     <row r="29">
@@ -20038,13 +20038,13 @@
         <v>1</v>
       </c>
       <c r="K29" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="L29" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="M29" t="n">
-        <v>77.8</v>
+        <v>78.09999999999999</v>
       </c>
     </row>
     <row r="30">
@@ -20074,7 +20074,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>blend(metis+fifa+nivel)</t>
+          <t>blend(metis+fifa+expert)</t>
         </is>
       </c>
       <c r="H30" t="n">
@@ -20090,7 +20090,7 @@
         <v>1.1</v>
       </c>
       <c r="L30" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="M30" t="n">
         <v>91.90000000000001</v>
@@ -20134,13 +20134,13 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="L31" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="M31" t="n">
-        <v>68.59999999999999</v>
+        <v>67.7</v>
       </c>
     </row>
     <row r="32">
@@ -20181,13 +20181,13 @@
         <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="L32" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="M32" t="n">
-        <v>62</v>
+        <v>61.3</v>
       </c>
     </row>
     <row r="33">
@@ -20228,13 +20228,13 @@
         <v>1</v>
       </c>
       <c r="K33" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L33" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="M33" t="n">
-        <v>33.1</v>
+        <v>34</v>
       </c>
     </row>
     <row r="34">
@@ -20275,13 +20275,13 @@
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="L34" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="M34" t="n">
-        <v>60.1</v>
+        <v>59.9</v>
       </c>
     </row>
     <row r="35">
@@ -20311,7 +20311,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>blend(metis+nivel)</t>
+          <t>blend(metis+expert)</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
@@ -20328,7 +20328,7 @@
         <v>1.2</v>
       </c>
       <c r="M35" t="n">
-        <v>48</v>
+        <v>48.3</v>
       </c>
     </row>
     <row r="36">
@@ -20372,10 +20372,10 @@
         <v>0.4</v>
       </c>
       <c r="L36" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="M36" t="n">
-        <v>55.5</v>
+        <v>55.9</v>
       </c>
     </row>
     <row r="37">
@@ -20416,13 +20416,13 @@
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>46.7</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="38">
@@ -20463,13 +20463,13 @@
         <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L38" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="M38" t="n">
-        <v>48.7</v>
+        <v>49.1</v>
       </c>
     </row>
     <row r="39">
@@ -20508,13 +20508,13 @@
         <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L39" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="M39" t="n">
-        <v>50.6</v>
+        <v>49.7</v>
       </c>
     </row>
     <row r="40">
@@ -20561,7 +20561,7 @@
         <v>0.7</v>
       </c>
       <c r="M40" t="n">
-        <v>44</v>
+        <v>43.9</v>
       </c>
     </row>
     <row r="41">
@@ -20605,10 +20605,10 @@
         <v>0.2</v>
       </c>
       <c r="L41" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="M41" t="n">
-        <v>48.4</v>
+        <v>48.9</v>
       </c>
     </row>
     <row r="42">
@@ -20655,7 +20655,7 @@
         <v>0.5</v>
       </c>
       <c r="M42" t="n">
-        <v>40.4</v>
+        <v>40.2</v>
       </c>
     </row>
     <row r="43">
@@ -20699,10 +20699,10 @@
         <v>0.1</v>
       </c>
       <c r="L43" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="M43" t="n">
-        <v>24.4</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="44">
@@ -20746,10 +20746,10 @@
         <v>0.2</v>
       </c>
       <c r="L44" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="M44" t="n">
-        <v>56</v>
+        <v>56.4</v>
       </c>
     </row>
     <row r="45">
@@ -20779,7 +20779,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>blend(metis+fifa+nivel)</t>
+          <t>blend(metis+fifa+expert)</t>
         </is>
       </c>
       <c r="H45" t="n">
@@ -20798,7 +20798,7 @@
         <v>0.3</v>
       </c>
       <c r="M45" t="n">
-        <v>29.8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46">
@@ -20840,10 +20840,10 @@
         <v>0.1</v>
       </c>
       <c r="L46" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="M46" t="n">
-        <v>32.5</v>
+        <v>32.9</v>
       </c>
     </row>
     <row r="47">
@@ -20885,10 +20885,10 @@
         <v>0.1</v>
       </c>
       <c r="L47" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="M47" t="n">
-        <v>54.3</v>
+        <v>53.6</v>
       </c>
     </row>
     <row r="48">
@@ -20933,7 +20933,7 @@
         <v>0.3</v>
       </c>
       <c r="M48" t="n">
-        <v>34</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="49">
@@ -20977,7 +20977,7 @@
         <v>0</v>
       </c>
       <c r="L49" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="M49" t="n">
         <v>11.4</v>

</xml_diff>